<commit_message>
docs: update test case documentation in Assignment 1 spreadsheet
</commit_message>
<xml_diff>
--- a/IT23641624_files/Assignment 1 - Test cases.xlsx
+++ b/IT23641624_files/Assignment 1 - Test cases.xlsx
@@ -1219,6 +1219,16 @@
           <t>ඔය server එක down වෙලා pen එකේ දාපන් files ටික.</t>
         </is>
       </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>English Digital Terms in Singlish</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
           <t>English Digital Terms in Singlish</t>
@@ -1249,6 +1259,11 @@
       <c r="D23" s="5" t="inlineStr">
         <is>
           <t>wifi password එක මොකක්ද?</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>UI Error</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">

</xml_diff>

<commit_message>
feat: complete Excel columns G & H for all 50 test cases
- Col G: 'Singlish input types covered' — correctly classified for all 50 rows
  using all 24 input types from Appendix 1
- Col H: 'Evidence or rationale for the input type covered' — detailed
  Evidence/Rationale entries for all 50 rows
- Fixed Neg_0049 mis-classification (was 'Isolated English Word Insertions',
  corrected to 'English digital terms in Singlish')
- Fixed 'Online Indentifiers' typo -> 'Online identifiers' in all affected rows
- Cleared 18 corrupted Actual output values that accidentally contained
  input-type strings from a previous buggy script run
- Updated both IT23641624_files/ and test_automation/ Excel copies
</commit_message>
<xml_diff>
--- a/IT23641624_files/Assignment 1 - Test cases.xlsx
+++ b/IT23641624_files/Assignment 1 - Test cases.xlsx
@@ -65,7 +65,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -77,6 +77,12 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -353,7 +359,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I51"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.130000000000001" customWidth="1" style="6" min="1" max="1"/>
     <col width="12.13" customWidth="1" style="6" min="2" max="2"/>
@@ -429,24 +435,20 @@
           <t>එහෙනම් අද අපි මොකක්ද කරන්නේ කියලා හිතුවේ ඔයා?</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>question forms</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="E2" s="0" t="n"/>
+      <c r="F2" s="0" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
         <is>
           <t>Question forms</t>
         </is>
       </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>Rationale: The sentence is asking a direct question about what to do today.</t>
+      <c r="H2" s="8" t="inlineStr">
+        <is>
+          <t>Rationale: The sentence ends with "oya?" — a direct question asking someone what they planned to do today, matching the question-form input type.</t>
         </is>
       </c>
     </row>
@@ -471,19 +473,19 @@
           <t>ඒගොල්ලෝ ගියාද එතකොට?</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="0" t="inlineStr">
         <is>
           <t>UI Error</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G3" s="7" t="inlineStr">
         <is>
           <t>Question forms</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>Rationale: The sentence structure ends with 'da', indicating an interrogative phrase.</t>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "giyada" — the "-da" suffix is the standard Singlish interrogative marker, forming a yes/no question.</t>
         </is>
       </c>
     </row>
@@ -508,24 +510,20 @@
           <t>ඔය වැඩේ මේ දැන්ම ඉවර කරලා දාන්න මචන්.</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>කොමන්ඩ් ෆෝර්ම්ස්</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="E4" s="0" t="n"/>
+      <c r="F4" s="0" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
         <is>
           <t>Command forms</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>Rationale: It is a direct instruction to finish a task immediately.</t>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>Rationale: "iwara karala danna" is a direct imperative instruction telling someone to finish the task immediately, matching the command-form input type.</t>
         </is>
       </c>
     </row>
@@ -550,19 +548,19 @@
           <t>ගිහින් එන්න ඉස්සෙල්ලා බලන්න.</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="0" t="inlineStr">
         <is>
           <t>UI Error</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G5" s="7" t="inlineStr">
         <is>
           <t>Command forms</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>Rationale: It is a command instructing someone to look before leaving.</t>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>Rationale: "ghin enna isella blanna" is a sequential command — go, come back, then look — structured as a direct instruction.</t>
         </is>
       </c>
     </row>
@@ -587,24 +585,20 @@
           <t>සුබ දවසක් වේවා හැමෝටම පරිස්සමින් යමන් එහෙනම්.</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>ග්රීටින්ග්ස්</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="E6" s="0" t="n"/>
+      <c r="F6" s="0" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
         <is>
           <t>Greetings</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: "suba dwasak wewa"</t>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "suba dwasak wewa" — a traditional Sinhala blessing phrase commonly used as a formal greeting or farewell.</t>
         </is>
       </c>
     </row>
@@ -629,19 +623,19 @@
           <t>ආයුබෝවන් මචන් කොහොමද උඹ?</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="0" t="inlineStr">
         <is>
           <t>UI Error</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>Greetings</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: "ayubowan"</t>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "ayubowan" — the standard Sinhala cultural greeting meaning "may you live long", directly matching the greetings input type.</t>
         </is>
       </c>
     </row>
@@ -666,24 +660,24 @@
           <t>පොඩ්ඩක් බලලා මට කියනවද වෙලා තියෙන දේ ටික?</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="0" t="inlineStr">
         <is>
           <t>Requests</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="F8" s="0" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
         <is>
           <t>Requests</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>Rationale: The user is politely asking someone to check and report back.</t>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>Rationale: "poddak blala mata kiyanawada" is a polite request asking someone to check and report back, matching the requests input type.</t>
         </is>
       </c>
     </row>
@@ -708,19 +702,19 @@
           <t>අනේ පොඩ්ඩක් ඒක දීපන්කෝ බන්.</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F9" s="0" t="inlineStr">
         <is>
           <t>UI Error</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G9" s="7" t="inlineStr">
         <is>
           <t>Requests</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: "ane pddk eka deepanko"</t>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "ane pddk eka deepanko" — "ane" and "deepanko" are request softeners in Singlish; the sentence is a polite ask to share something.</t>
         </is>
       </c>
     </row>
@@ -745,24 +739,24 @@
           <t>ඒක නම් සිරා කතාව එහෙමම තමා වෙච්චේ එදා.</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="0" t="inlineStr">
         <is>
           <t>රෙපන්ස්</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="F10" s="0" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
         <is>
           <t>Responses</t>
         </is>
       </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>Rationale: The sentence is an affirmative response confirming a previous statement.</t>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>Rationale: "eka nam sira kathaawa ehemama tama wechcha" is an affirmative response confirming that something happened exactly as discussed, matching the responses input type.</t>
         </is>
       </c>
     </row>
@@ -787,19 +781,19 @@
           <t>ඔව් ඔව් ඒක හරි මම එදා ගියා.</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F11" s="0" t="inlineStr">
         <is>
           <t>UI Error</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="G11" s="7" t="inlineStr">
         <is>
           <t>Responses</t>
         </is>
       </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: "ow ow eka hri"</t>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "ow ow eka hri" — "ow" is the Singlish affirmative particle (yes), and its repetition with "eka hri" confirms agreement, matching the responses input type.</t>
         </is>
       </c>
     </row>
@@ -824,24 +818,24 @@
           <t>උඹ හෙමින් හෙමින් වරෙන්කෝ හදිස්සි වෙන්නේ නැතුව.</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="0" t="inlineStr">
         <is>
           <t>Repeated Words</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>Repeated Words</t>
-        </is>
-      </c>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: "hemin hemin"</t>
+      <c r="F12" s="0" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>Repeated words</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "hemin hemin" — the word "hemin" (slowly/carefully) is repeated consecutively, a common Singlish emphasis pattern matching the repeated-words input type.</t>
         </is>
       </c>
     </row>
@@ -866,19 +860,19 @@
           <t>ටිකක් ටිකක් දීලා බලන්න.</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F13" s="0" t="inlineStr">
         <is>
           <t>UI Error</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>Repeated Words</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: "tkak tkak"</t>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>Repeated words</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "tkak tkak" — "tkak" (a bit) is repeated, a typical Singlish reduplication pattern used for emphasis, matching the repeated-words input type.</t>
         </is>
       </c>
     </row>
@@ -903,24 +897,24 @@
           <t>එහෙනම්, අපි හෙට සෙට් වෙමු නේද? අනිවා!! ගින්දර..</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" s="0" t="inlineStr">
         <is>
           <t>ඉන්පුට්ස් with Punctuation Marks</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>Inputs with Punctuation Marks</t>
-        </is>
-      </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>Rationale: The input uses commas, question marks, and multiple exclamation points.</t>
+      <c r="F14" s="0" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>Rationale: The input uses a comma, question mark, and double exclamation ("neda?", "aniwa!!") in one sentence — multiple punctuation types within a single conversational Singlish input.</t>
         </is>
       </c>
     </row>
@@ -945,19 +939,19 @@
           <t>මොකක්ද බන් ඒ?! කියපන්කෝ...</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F15" s="0" t="inlineStr">
         <is>
           <t>UI Error</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>Inputs with Punctuation Marks</t>
-        </is>
-      </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>Rationale: The input features consecutive punctuation marks like '?!' and '...' .</t>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with punctuation marks</t>
+        </is>
+      </c>
+      <c r="H15" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "?!" and "..." — the input contains mixed consecutive punctuation (interrobang-style "?!" and ellipsis "..."), testing how the translator handles non-standard punctuation sequences.</t>
         </is>
       </c>
     </row>
@@ -982,24 +976,20 @@
           <t>මං නම් කියන්නේ ඔය වැඩේ කරන්න එපා කියලා එයාට.</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>රෝමාණිකරණය / ස්පීලිංගේ විකෘති</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G16" s="5" t="inlineStr">
-        <is>
-          <t>Romanization / Spelling Variants</t>
-        </is>
-      </c>
-      <c r="H16" s="5" t="inlineStr">
-        <is>
-          <t>Rationale: The word 'wedee' is written with a double 'e' and 'kranna' omits the 'a'.</t>
+      <c r="E16" s="0" t="n"/>
+      <c r="F16" s="0" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>Romanization / Spelling variants</t>
+        </is>
+      </c>
+      <c r="H16" s="8" t="inlineStr">
+        <is>
+          <t>Rationale: "wedee" uses an extra vowel (double-e) as a non-standard spelling variant of "wede", representing a phonetic spelling deviation from standard Singlish romanization.</t>
         </is>
       </c>
     </row>
@@ -1024,19 +1014,19 @@
           <t>මගේ පොත දීලා යන්න එන්න.</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F17" s="0" t="inlineStr">
         <is>
           <t>UI Error</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
-        <is>
-          <t>Romanization / Spelling Variants</t>
-        </is>
-      </c>
-      <c r="H17" s="5" t="inlineStr">
-        <is>
-          <t>Rationale: Words are heavily abbreviated by dropping vowels (e.g., 'mge', 'ptha', 'ynn').</t>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>Romanization / Spelling variants</t>
+        </is>
+      </c>
+      <c r="H17" s="8" t="inlineStr">
+        <is>
+          <t>Rationale: "ptha", "ynn", "enna" are heavily abbreviated variants of "putha", "yanna", "enna" — dropping vowels mid-word is a common informal Singlish romanization pattern.</t>
         </is>
       </c>
     </row>
@@ -1061,24 +1051,20 @@
           <t>මගේ phone එක කැඩිලා වෙන එකක් ගන්න ඕනේ දැන්.</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>ඉසෝලated English Word Insertions in Singlish</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G18" s="5" t="inlineStr">
-        <is>
-          <t>Isolated English Word Insertions in Singlish</t>
-        </is>
-      </c>
-      <c r="H18" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: The single English word "phone" is used mid-sentence.</t>
+      <c r="E18" s="0" t="n"/>
+      <c r="F18" s="0" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>Isolated English word insertions in Singlish</t>
+        </is>
+      </c>
+      <c r="H18" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "phone" — a single English noun is inserted into an otherwise Singlish sentence ("mage phone eka"), representing the isolated-English-word insertion input type.</t>
         </is>
       </c>
     </row>
@@ -1103,19 +1089,19 @@
           <t>හෙට ලොකු meeting එකක් තියෙනවා.</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F19" s="0" t="inlineStr">
         <is>
           <t>UI Error</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>Isolated English Word Insertions in Singlish</t>
-        </is>
-      </c>
-      <c r="H19" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: The single English word "meeting" is inserted.</t>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>Isolated English word insertions in Singlish</t>
+        </is>
+      </c>
+      <c r="H19" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "meeting" — a single English noun is embedded in a Singlish sentence ("loku meeting ekak tynwa"), representing an isolated English word insertion.</t>
         </is>
       </c>
     </row>
@@ -1140,24 +1126,24 @@
           <t>අපි end of the day කොහොමහරි project එක දෙමු.</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E20" s="0" t="inlineStr">
         <is>
           <t>Multi-Word English Phrases in Singlish</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G20" s="5" t="inlineStr">
-        <is>
-          <t>Multi-Word English Phrases in Singlish</t>
-        </is>
-      </c>
-      <c r="H20" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: The phrase "end of the day" is used.</t>
+      <c r="F20" s="0" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>Multi-word English phrases in Singlish</t>
+        </is>
+      </c>
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "end of the day" — a complete multi-word English idiomatic phrase is used inline within a Singlish sentence, matching the multi-word English phrase input type.</t>
         </is>
       </c>
     </row>
@@ -1182,19 +1168,19 @@
           <t>ඒක නම් out of the box හිතලා කරපු වැඩක් තමා.</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="F21" s="0" t="inlineStr">
         <is>
           <t>UI Error</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>Multi-Word English Phrases in Singlish</t>
-        </is>
-      </c>
-      <c r="H21" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: The phrase "out of the box" is used.</t>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>Multi-word English phrases in Singlish</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "out of the box" — a complete multi-word English idiomatic expression is embedded in a Singlish sentence, matching the multi-word English phrase input type.</t>
         </is>
       </c>
     </row>
@@ -1219,24 +1205,24 @@
           <t>ඔය server එක down වෙලා pen එකේ දාපන් files ටික.</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E22" s="0" t="inlineStr">
         <is>
           <t>English Digital Terms in Singlish</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G22" s="5" t="inlineStr">
-        <is>
-          <t>English Digital Terms in Singlish</t>
-        </is>
-      </c>
-      <c r="H22" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: The digital terms "server", "down", and "files" are present.</t>
+      <c r="F22" s="0" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>English digital terms in Singlish</t>
+        </is>
+      </c>
+      <c r="H22" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "server", "down", "fix" — three English digital/technical terms are embedded within a conversational Singlish sentence, matching the English digital terms input type.</t>
         </is>
       </c>
     </row>
@@ -1261,19 +1247,19 @@
           <t>wifi password එක මොකක්ද?</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F23" s="0" t="inlineStr">
         <is>
           <t>UI Error</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr">
-        <is>
-          <t>English Digital Terms in Singlish</t>
-        </is>
-      </c>
-      <c r="H23" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: The digital terms "wifi" and "password" are present.</t>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>English digital terms in Singlish</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "wifi", "password" — two common English digital terms are used in a Singlish question, matching the English digital terms input type.</t>
         </is>
       </c>
     </row>
@@ -1298,24 +1284,24 @@
           <t>උඹ telegram එකෙන් එවන්න ඒක ලේසි whatsapp වලට.</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E24" s="0" t="inlineStr">
         <is>
           <t>Platform/App Names in Singlish</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G24" s="5" t="inlineStr">
-        <is>
-          <t>Platform/App Names in Singlish</t>
-        </is>
-      </c>
-      <c r="H24" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: "telegram" and "watsapp"</t>
+      <c r="F24" s="0" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>Platform / app names in Singlish</t>
+        </is>
+      </c>
+      <c r="H24" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "telegram", "watsapp" — two social media / messaging platform names are referenced inline in a Singlish sentence, matching the platform/app names input type.</t>
         </is>
       </c>
     </row>
@@ -1340,19 +1326,19 @@
           <t>instagram post එක දාන්න.</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="F25" s="0" t="inlineStr">
         <is>
           <t>UI Error</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>Platform/App Names in Singlish</t>
-        </is>
-      </c>
-      <c r="H25" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: "instagram"</t>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>Platform / app names in Singlish</t>
+        </is>
+      </c>
+      <c r="H25" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "instagram" — the name of a major social media platform is used directly in a Singlish command, matching the platform/app names input type.</t>
         </is>
       </c>
     </row>
@@ -1377,24 +1363,24 @@
           <t>මම CV එක එවන්නම් පුළුවන් තරම් ASAP බලන්න.</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E26" s="0" t="inlineStr">
         <is>
           <t>English Abbreviations/Acronyms in Singlish</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G26" s="5" t="inlineStr">
-        <is>
-          <t>English Abbreviations/Acronyms in Singlish</t>
-        </is>
-      </c>
-      <c r="H26" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: "CV" and "ASAP"</t>
+      <c r="F26" s="0" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>English abbreviations / acronyms in Singlish</t>
+        </is>
+      </c>
+      <c r="H26" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "CV" (curriculum vitae) and "ASAP" (as soon as possible) — two English acronyms are used in a single Singlish sentence, matching the abbreviations/acronyms input type.</t>
         </is>
       </c>
     </row>
@@ -1419,19 +1405,19 @@
           <t>මට ETA එක කියන්න පුළුවන්ද?</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="F27" s="0" t="inlineStr">
         <is>
           <t>UI Error</t>
         </is>
       </c>
-      <c r="G27" s="5" t="inlineStr">
-        <is>
-          <t>English Abbreviations/Acronyms in Singlish</t>
-        </is>
-      </c>
-      <c r="H27" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: "ETA"</t>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>English abbreviations / acronyms in Singlish</t>
+        </is>
+      </c>
+      <c r="H27" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "ETA" (estimated time of arrival) — an English acronym is inserted in a Singlish question, matching the abbreviations/acronyms input type.</t>
         </is>
       </c>
     </row>
@@ -1456,24 +1442,20 @@
           <t>හෙට මීට වඩා ටිකක් ලොකු lab එකකට යන්න වෙනවා.</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>English Clipped Forms in Singlish</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G28" s="5" t="inlineStr">
-        <is>
-          <t>English Clipped Forms in Singlish</t>
-        </is>
-      </c>
-      <c r="H28" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: "lab" is used instead of laboratory.</t>
+      <c r="E28" s="0" t="n"/>
+      <c r="F28" s="0" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>English clipped forms in Singlish</t>
+        </is>
+      </c>
+      <c r="H28" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "lab" — a clipped form of "laboratory" is used in a Singlish sentence, matching the English clipped forms input type.</t>
         </is>
       </c>
     </row>
@@ -1498,19 +1480,19 @@
           <t>exam එකක් තියෙනවා හෙට උදේම.</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="F29" s="0" t="inlineStr">
         <is>
           <t>UI Error</t>
         </is>
       </c>
-      <c r="G29" s="5" t="inlineStr">
-        <is>
-          <t>English Clipped Forms in Singlish</t>
-        </is>
-      </c>
-      <c r="H29" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: "exam" is used instead of examination.</t>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>English clipped forms in Singlish</t>
+        </is>
+      </c>
+      <c r="H29" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "exam" — a clipped form of "examination" is embedded in a Singlish sentence, matching the English clipped forms input type.</t>
         </is>
       </c>
     </row>
@@ -1535,24 +1517,20 @@
           <t>හෙට නුගේගොඩ junction එක ගාව මං ඉන්නම් වේලාසන.</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Place Names Embedded in Singlish</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G30" s="5" t="inlineStr">
-        <is>
-          <t>Place Names Embedded in Singlish</t>
-        </is>
-      </c>
-      <c r="H30" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: The location "nugegoda" is explicitly mentioned.</t>
+      <c r="E30" s="0" t="n"/>
+      <c r="F30" s="0" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>Place names embedded in Singlish</t>
+        </is>
+      </c>
+      <c r="H30" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "nugegoda junction" — the Sri Lankan place name "Nugegoda" is directly embedded in a Singlish sentence to describe a meeting location, matching the place names input type.</t>
         </is>
       </c>
     </row>
@@ -1577,19 +1555,19 @@
           <t>mt lavinia පැත්තේ යමු අද.</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F31" s="0" t="inlineStr">
         <is>
           <t>UI Error</t>
         </is>
       </c>
-      <c r="G31" s="5" t="inlineStr">
-        <is>
-          <t>Place Names Embedded in Singlish</t>
-        </is>
-      </c>
-      <c r="H31" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: The location "mt lavinia" is explicitly mentioned.</t>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>Place names embedded in Singlish</t>
+        </is>
+      </c>
+      <c r="H31" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "mt lavinia" — the Sri Lankan coastal locality "Mt. Lavinia" is embedded in a Singlish suggestion, matching the place names input type.</t>
         </is>
       </c>
     </row>
@@ -1614,24 +1592,20 @@
           <t>ඒ වැඩේ චාමර අයියට දීලා තියෙන්නේ බය වෙන්න එපා.</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Person Names Embedded in Singlish</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G32" s="5" t="inlineStr">
-        <is>
-          <t>Person Names Embedded in Singlish</t>
-        </is>
-      </c>
-      <c r="H32" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: The person name "chamara" is used.</t>
+      <c r="E32" s="0" t="n"/>
+      <c r="F32" s="0" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>Person names embedded in Singlish</t>
+        </is>
+      </c>
+      <c r="H32" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "chamara aiya" — the person name "Chamara" with the kinship title "aiya" (elder brother) is embedded in a Singlish sentence, matching the person names input type.</t>
         </is>
       </c>
     </row>
@@ -1656,19 +1630,19 @@
           <t>නිමල් මචන් මොකද කරන්නේ?</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F33" s="0" t="inlineStr">
         <is>
           <t>UI Error</t>
         </is>
       </c>
-      <c r="G33" s="5" t="inlineStr">
-        <is>
-          <t>Person Names Embedded in Singlish</t>
-        </is>
-      </c>
-      <c r="H33" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: The person name "nimal" is used.</t>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>Person names embedded in Singlish</t>
+        </is>
+      </c>
+      <c r="H33" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "nimal" — the person name "Nimal" is used as the subject of a Singlish question, matching the person names input type.</t>
         </is>
       </c>
     </row>
@@ -1693,24 +1667,20 @@
           <t>මට 10ක් වත් එවනවද අර සල්ලි වලින් අඩු කරලා.</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>ඉන්පුට්ස් with Numbers and Numeric Suffixes</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G34" s="5" t="inlineStr">
-        <is>
-          <t>Inputs with Numbers and Numeric Suffixes</t>
-        </is>
-      </c>
-      <c r="H34" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: "10k" combines a number with a Singlish suffix.</t>
+      <c r="E34" s="0" t="n"/>
+      <c r="F34" s="0" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with numbers and numeric suffixes</t>
+        </is>
+      </c>
+      <c r="H34" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "10k" — the numeral "10" is combined with the Singlish/English suffix "k" (thousand), forming a mixed numeric token, matching the numbers and numeric suffixes input type.</t>
         </is>
       </c>
     </row>
@@ -1735,19 +1705,19 @@
           <t>උඹ 3වෙනි පේළියේ ඉන්න.</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F35" s="0" t="inlineStr">
         <is>
           <t>UI Error</t>
         </is>
       </c>
-      <c r="G35" s="5" t="inlineStr">
-        <is>
-          <t>Inputs with Numbers and Numeric Suffixes</t>
-        </is>
-      </c>
-      <c r="H35" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: "3weni" combines a number with a Singlish suffix.</t>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with numbers and numeric suffixes</t>
+        </is>
+      </c>
+      <c r="H35" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "3weni" — the numeral "3" is combined with the Sinhala ordinal suffix "weni" (third), forming a numeric–suffix token, matching the numbers and numeric suffixes input type.</t>
         </is>
       </c>
     </row>
@@ -1772,24 +1742,20 @@
           <t>අර රු 5000 දීපන්කෝ අද හවසට ආපහු දෙන්නම්.</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Inputs with Currency</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G36" s="5" t="inlineStr">
-        <is>
-          <t>Inputs with Currency</t>
-        </is>
-      </c>
-      <c r="H36" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: "rs 5000"</t>
+      <c r="E36" s="0" t="n"/>
+      <c r="F36" s="0" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G36" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with currency</t>
+        </is>
+      </c>
+      <c r="H36" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "rs 5000" — the Sri Lankan currency abbreviation "rs" (rupees) is used with a numeral amount in a Singlish sentence, matching the currency input type.</t>
         </is>
       </c>
     </row>
@@ -1814,19 +1780,19 @@
           <t>$50 කියන්නේ කීයද දැන්?</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F37" s="0" t="inlineStr">
         <is>
           <t>UI Error</t>
         </is>
       </c>
-      <c r="G37" s="5" t="inlineStr">
-        <is>
-          <t>Inputs with Currency</t>
-        </is>
-      </c>
-      <c r="H37" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: "$50"</t>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with currency</t>
+        </is>
+      </c>
+      <c r="H37" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "$50" — the US dollar symbol "$" is used with a numeral in a Singlish question, matching the currency input type.</t>
         </is>
       </c>
     </row>
@@ -1851,24 +1817,20 @@
           <t>අපිට හෙට 10.30am වෙද්දී office ඉන්න පුළුවන්ද කියලා දාපන්.</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Inputs with Time formats</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G38" s="5" t="inlineStr">
-        <is>
-          <t>Inputs with Time Formats</t>
-        </is>
-      </c>
-      <c r="H38" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: "10.30am"</t>
+      <c r="E38" s="0" t="n"/>
+      <c r="F38" s="0" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with time formats</t>
+        </is>
+      </c>
+      <c r="H38" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "10.30am" — a 12-hour clock time with AM/PM suffix is embedded in a Singlish sentence, matching the time formats input type.</t>
         </is>
       </c>
     </row>
@@ -1893,19 +1855,19 @@
           <t>හවස් 5pm වෙනකොට මං එන්නම්.</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F39" s="0" t="inlineStr">
         <is>
           <t>UI Error</t>
         </is>
       </c>
-      <c r="G39" s="5" t="inlineStr">
-        <is>
-          <t>Inputs with Time Formats</t>
-        </is>
-      </c>
-      <c r="H39" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: "5pm"</t>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with time formats</t>
+        </is>
+      </c>
+      <c r="H39" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "5pm" — a 12-hour clock time with a PM suffix is used in a Singlish statement, matching the time formats input type.</t>
         </is>
       </c>
     </row>
@@ -1930,24 +1892,20 @@
           <t>මගේ birthday එක තියෙන්නේ 2026-10-15 මතක තියා ගනින්.</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>ඉන්පුට්ස් විත් ඩේට්ස්</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G40" s="5" t="inlineStr">
-        <is>
-          <t>Inputs with Dates</t>
-        </is>
-      </c>
-      <c r="H40" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: "2026-10-15"</t>
+      <c r="E40" s="0" t="n"/>
+      <c r="F40" s="0" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G40" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with dates</t>
+        </is>
+      </c>
+      <c r="H40" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "2026-10-15" — an ISO 8601 formatted date (YYYY-MM-DD) is embedded in a Singlish sentence, matching the dates input type.</t>
         </is>
       </c>
     </row>
@@ -1972,19 +1930,19 @@
           <t>oct 15 තමා වැඩේ ඉවර.</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F41" s="0" t="inlineStr">
         <is>
           <t>UI Error</t>
         </is>
       </c>
-      <c r="G41" s="5" t="inlineStr">
-        <is>
-          <t>Inputs with Dates</t>
-        </is>
-      </c>
-      <c r="H41" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: "oct 15"</t>
+      <c r="G41" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with dates</t>
+        </is>
+      </c>
+      <c r="H41" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "oct 15" — an abbreviated month name followed by a day number is used in a Singlish sentence, matching the dates input type.</t>
         </is>
       </c>
     </row>
@@ -2009,24 +1967,20 @@
           <t>ගෙදර ඉඳලා town එකට 5km තියෙනවා පයින් යමු අපි.</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>ඉන්පුට්ස් with Unit of Measurements</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G42" s="5" t="inlineStr">
-        <is>
-          <t>Inputs with Unit of Measurements</t>
-        </is>
-      </c>
-      <c r="H42" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: "5km"</t>
+      <c r="E42" s="0" t="n"/>
+      <c r="F42" s="0" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G42" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with units of measurement</t>
+        </is>
+      </c>
+      <c r="H42" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "5km" — the metric distance unit "km" (kilometres) is combined with a numeral in a Singlish sentence, matching the units of measurement input type.</t>
         </is>
       </c>
     </row>
@@ -2051,19 +2005,19 @@
           <t>පිටි 2kg ගෙන්න ඇතුව.</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F43" s="0" t="inlineStr">
         <is>
           <t>UI Error</t>
         </is>
       </c>
-      <c r="G43" s="5" t="inlineStr">
-        <is>
-          <t>Inputs with Unit of Measurements</t>
-        </is>
-      </c>
-      <c r="H43" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: "2kg"</t>
+      <c r="G43" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with units of measurement</t>
+        </is>
+      </c>
+      <c r="H43" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "2kg" — the metric weight unit "kg" (kilograms) is combined with a numeral in a Singlish command, matching the units of measurement input type.</t>
         </is>
       </c>
     </row>
@@ -2088,24 +2042,20 @@
           <t>සුපිරි බන් උඹ නම් පට්ට ඩයල් එකක් නේ සිරාවටම.</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>ඉන්පුට්ස් විත් ස්ලන්ග් and Casual Phrasing</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G44" s="5" t="inlineStr">
-        <is>
-          <t>Inputs with Slang and Casual Phrasing</t>
-        </is>
-      </c>
-      <c r="H44" s="5" t="inlineStr">
-        <is>
-          <t>Rationale: Uses heavy colloquial slang like "patta dial" and "sirawatama".</t>
+      <c r="E44" s="0" t="n"/>
+      <c r="F44" s="0" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G44" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with slang and casual phrasing</t>
+        </is>
+      </c>
+      <c r="H44" s="8" t="inlineStr">
+        <is>
+          <t>Rationale: Uses heavy Singlish slang — "patta dial" (awesome call/move), "sirawatama" (absolutely perfectly), "bn" (bana/friend) — all informal colloquial tokens matching the slang and casual phrasing input type.</t>
         </is>
       </c>
     </row>
@@ -2130,19 +2080,19 @@
           <t>ඌට මල පැනලා තියෙන්නේ.</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F45" s="0" t="inlineStr">
         <is>
           <t>UI Error</t>
         </is>
       </c>
-      <c r="G45" s="5" t="inlineStr">
-        <is>
-          <t>Inputs with Slang and Casual Phrasing</t>
-        </is>
-      </c>
-      <c r="H45" s="5" t="inlineStr">
-        <is>
-          <t>Rationale: Uses the informal idiom "mala panala".</t>
+      <c r="G45" s="7" t="inlineStr">
+        <is>
+          <t>Inputs with slang and casual phrasing</t>
+        </is>
+      </c>
+      <c r="H45" s="8" t="inlineStr">
+        <is>
+          <t>Rationale: "mala panala" is an idiomatic Singlish slang phrase meaning something went very wrong/crazy; it is an informal colloquial expression matching the slang and casual phrasing input type.</t>
         </is>
       </c>
     </row>
@@ -2167,24 +2117,20 @@
           <t>ඔය වැඩේ ගැන ඉගෙන ගන්න www.w3schools.com යමන්.</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>Online Indentifiers in Singlish</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G46" s="5" t="inlineStr">
-        <is>
-          <t>Online Indentifiers in Singlish</t>
-        </is>
-      </c>
-      <c r="H46" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: Contains the URL "www.w3schools.com"</t>
+      <c r="E46" s="0" t="n"/>
+      <c r="F46" s="0" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G46" s="7" t="inlineStr">
+        <is>
+          <t>Online identifiers in Singlish</t>
+        </is>
+      </c>
+      <c r="H46" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "www.w3schools.com" — a full URL is embedded mid-sentence in a Singlish statement, matching the online identifiers input type.</t>
         </is>
       </c>
     </row>
@@ -2209,19 +2155,19 @@
           <t>@nimal123 tag කරලා දාපන්.</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="F47" s="0" t="inlineStr">
         <is>
           <t>UI Error</t>
         </is>
       </c>
-      <c r="G47" s="5" t="inlineStr">
-        <is>
-          <t>Online Indentifiers in Singlish</t>
-        </is>
-      </c>
-      <c r="H47" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: Contains the handle "@nimal123"</t>
+      <c r="G47" s="7" t="inlineStr">
+        <is>
+          <t>Online identifiers in Singlish</t>
+        </is>
+      </c>
+      <c r="H47" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "@nimal123" — a social media handle (@ + username) is used in a Singlish command, matching the online identifiers input type.</t>
         </is>
       </c>
     </row>
@@ -2246,24 +2192,20 @@
           <t>ඒක අහලා මට හිනා ගිහින් පණ ගියා 😂 මාර සීන් එක.</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>Inputs Containing Emojis</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G48" s="5" t="inlineStr">
-        <is>
-          <t>Inputs Containing Emojis</t>
-        </is>
-      </c>
-      <c r="H48" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: Contains the 😂 emoji.</t>
+      <c r="E48" s="0" t="n"/>
+      <c r="F48" s="0" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G48" s="7" t="inlineStr">
+        <is>
+          <t>Inputs containing emojis</t>
+        </is>
+      </c>
+      <c r="H48" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: 😂 — the "face with tears of joy" emoji is embedded mid-sentence within a Singlish statement, matching the emojis input type.</t>
         </is>
       </c>
     </row>
@@ -2288,19 +2230,19 @@
           <t>congratzz මචන් 🎉💪 එළ.</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
+      <c r="F49" s="0" t="inlineStr">
         <is>
           <t>UI Error</t>
         </is>
       </c>
-      <c r="G49" s="5" t="inlineStr">
-        <is>
-          <t>Inputs Containing Emojis</t>
-        </is>
-      </c>
-      <c r="H49" s="5" t="inlineStr">
-        <is>
-          <t>Evidence: Contains the 🎉 and 💪 emojis.</t>
+      <c r="G49" s="7" t="inlineStr">
+        <is>
+          <t>Inputs containing emojis</t>
+        </is>
+      </c>
+      <c r="H49" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: 🎉💪 — a "party popper" and "flexed bicep" emoji are used together in a short Singlish congratulatory message, matching the emojis input type.</t>
         </is>
       </c>
     </row>
@@ -2325,24 +2267,20 @@
           <t>frontend එක build කරද්දි error එකක් ආවා පොඩ්ඩක් බලන්න.</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>ඉසෝලated English Word Insertions in Singlish</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G50" s="5" t="inlineStr">
-        <is>
-          <t>Isolated English Word Insertions in Singlish</t>
-        </is>
-      </c>
-      <c r="H50" s="5" t="inlineStr">
-        <is>
-          <t>Rationale: Testing technical developer jargon mixed into conversational text.</t>
+      <c r="E50" s="0" t="n"/>
+      <c r="F50" s="0" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G50" s="7" t="inlineStr">
+        <is>
+          <t>English digital terms in Singlish</t>
+        </is>
+      </c>
+      <c r="H50" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: "frontend", "build", "error" — three technical software development terms are embedded in a conversational Singlish sentence, matching the English digital terms input type.</t>
         </is>
       </c>
     </row>
@@ -2367,24 +2305,20 @@
           <t>හැමෝම එකතු වෙලා මේ වැඩේ ලේසියෙන් ගොඩ දාගමු කොල්ලෝ.</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>රෝමාණිකරණය / ස්පීලිංගේ විකෘති</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G51" s="5" t="inlineStr">
-        <is>
-          <t>Romanization / Spelling Variants</t>
-        </is>
-      </c>
-      <c r="H51" s="5" t="inlineStr">
-        <is>
-          <t>Rationale: Testing extreme abbreviation ('hmoma', 'wdee', 'dgamu') commonly found in group chats.</t>
+      <c r="E51" s="0" t="n"/>
+      <c r="F51" s="0" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G51" s="7" t="inlineStr">
+        <is>
+          <t>Romanization / Spelling variants</t>
+        </is>
+      </c>
+      <c r="H51" s="8" t="inlineStr">
+        <is>
+          <t>Rationale: "hmoma" (for "hamoma"), "wdee" (for "wede"), "dgamu" (for "dagamu") — extreme vowel-dropping abbreviations typical of fast Singlish group-chat typing, matching the romanization/spelling variants input type.</t>
         </is>
       </c>
     </row>

</xml_diff>